<commit_message>
Do final corrections of second term - taller 6
</commit_message>
<xml_diff>
--- a/06-normatividad/checklist-cliente.xlsx
+++ b/06-normatividad/checklist-cliente.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>El formulario único de inscripción exige la autorización expresa del propio usuario (pregunta 1, obligatoria) para registrarlo en Koha y en la Llave del Saber; la respuesta queda registrada en Microsoft Forms.</t>
+          <t>El formulario único de inscripción exige la autorización expresa del propio usuario (pregunta 1, obligatoria) para registrarlo en Koha y en la Llave del Saber; la respuesta queda registrada en Microsoft Forms. Formulario publicado el 1 de octubre de 2026. Evidencia: evidencia/02-pregunta-1-autorizacion.png, evidencia/formulario-inscripcion-2026-10-01.pdf.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>El aviso del formulario identifica a la Alcaldía como Responsable, incluye su teléfono, las finalidades, los derechos del art. 8, los canales oficiales y el enlace a la política publicada.</t>
+          <t>El aviso del formulario identifica a la Alcaldía como Responsable, incluye su teléfono, las finalidades, los derechos del art. 8, los canales oficiales y el enlace a la política publicada (formulario publicado el 1 de octubre de 2026). Evidencia: evidencia/01-aviso-de-privacidad.png, evidencia/02-pregunta-1-autorizacion.png.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Existe una autorización separada para datos sensibles (pregunta 2) y grupo étnico permite "No responde", pero discapacidad es obligatoria sin opción de no responder y elegir "No autorizo" en la pregunta 2 impide la inscripción.</t>
+          <t>Existe una autorización separada para datos sensibles (pregunta 2) y grupo étnico permite "No responde", pero discapacidad es obligatoria sin opción de no responder y elegir "No autorizo" en la pregunta 2 impide la inscripción. Evidencia: evidencia/03-pregunta-2-datos-sensibles.png.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>El aviso anuncia la confirmación presencial con el acudiente de las inscripciones de menores hechas en línea, pero no se evidenció el procedimiento; el formulario solo pide nombre, teléfono y parentesco del adulto.</t>
+          <t>El aviso anuncia la confirmación presencial con el acudiente de las inscripciones de menores hechas en línea, pero no se evidenció el procedimiento; el formulario solo pide nombre, teléfono y parentesco del adulto. Evidencia: evidencia/01-aviso-de-privacidad.png.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>La política define canales y plazos (num. 11) y el aviso del formulario remite a esos canales oficiales (correo institucional, Ventanilla Única y PQRSD) con los mismos plazos.</t>
+          <t>La política define canales y plazos (num. 11) y el aviso del formulario remite a esos canales oficiales (correo institucional, Ventanilla Única y PQRSD) con los mismos plazos. Evidencia: evidencia/02-pregunta-1-autorizacion.png.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>El aviso ya justifica estudios, ocupación, grupo étnico y discapacidad; sexo al nacer, hábitos de lectura y estrato (exigido por la Llave del Saber) no tienen finalidad informada.</t>
+          <t>El aviso ya justifica estudios, ocupación, grupo étnico y discapacidad; sexo al nacer, hábitos de lectura y estrato (exigido por la Llave del Saber) no tienen finalidad informada. Evidencia: evidencia/formulario-inscripcion-2026-10-01.pdf.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">

</xml_diff>